<commit_message>
Backup local changes before pull
</commit_message>
<xml_diff>
--- a/Unified_PDF_Platform/unified_outputs/Guardian Rocca Feb-25 Inv 2_invoice.xlsx
+++ b/Unified_PDF_Platform/unified_outputs/Guardian Rocca Feb-25 Inv 2_invoice.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P75"/>
+  <dimension ref="A1:Q83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,6 +507,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>PRICING_ADJUSTMENT</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_AMOUNT</t>
         </is>
       </c>
     </row>
@@ -555,6 +560,9 @@
         <v>7.5</v>
       </c>
       <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -601,6 +609,9 @@
         <v>5</v>
       </c>
       <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -647,6 +658,9 @@
         <v>7.5</v>
       </c>
       <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -693,6 +707,9 @@
         <v>32</v>
       </c>
       <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -739,6 +756,9 @@
         <v>11.22</v>
       </c>
       <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -785,6 +805,9 @@
         <v>-53.53</v>
       </c>
       <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -831,6 +854,9 @@
         <v>-33.76</v>
       </c>
       <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -877,6 +903,9 @@
         <v>2.85</v>
       </c>
       <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -921,6 +950,9 @@
         <v>-2.75</v>
       </c>
       <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -965,6 +997,9 @@
         <v>-17.31</v>
       </c>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1009,6 +1044,9 @@
         <v>-7.42</v>
       </c>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1053,6 +1091,9 @@
         <v>-1.24</v>
       </c>
       <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1097,6 +1138,9 @@
         <v>-0.53</v>
       </c>
       <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1141,6 +1185,9 @@
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1189,6 +1236,9 @@
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1237,6 +1287,9 @@
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1281,6 +1334,9 @@
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1329,6 +1385,9 @@
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1377,6 +1436,9 @@
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1421,6 +1483,9 @@
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1469,6 +1534,9 @@
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1517,6 +1585,9 @@
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1561,6 +1632,9 @@
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1609,6 +1683,9 @@
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1653,6 +1730,9 @@
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1697,6 +1777,9 @@
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1741,6 +1824,9 @@
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1785,6 +1871,9 @@
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1833,6 +1922,9 @@
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1877,10 +1969,13 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>12.53</v>
+        <v>7.42</v>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1901,12 +1996,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fayson</t>
+          <t>Crouch</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Bryonne</t>
+          <t>TherralR</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1915,16 +2010,23 @@
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
       <c r="N32" t="n">
-        <v>2.5</v>
+        <v>12.53</v>
       </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1959,20 +2061,19 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
-        <v>17.31</v>
+        <v>2.5</v>
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2007,20 +2108,23 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
-          <t>VISION</t>
+          <t>DENTAL</t>
         </is>
       </c>
       <c r="N34" t="n">
-        <v>8.279999999999999</v>
+        <v>17.31</v>
       </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2041,12 +2145,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Gerhart</t>
+          <t>Fayson</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PaulR</t>
+          <t>Bryonne</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -2055,16 +2159,23 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
       <c r="N35" t="n">
-        <v>2.75</v>
+        <v>7.42</v>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2085,12 +2196,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Gerhart</t>
+          <t>Fayson</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>PaulR</t>
+          <t>Bryonne</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -2099,20 +2210,23 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
-          <t>DENTAL</t>
+          <t>VISION</t>
         </is>
       </c>
       <c r="N36" t="n">
-        <v>17.31</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2147,20 +2261,19 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>VISION</t>
-        </is>
-      </c>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="n">
-        <v>15.88</v>
+        <v>2.75</v>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2181,12 +2294,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Graves</t>
+          <t>Gerhart</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>CarsonJ</t>
+          <t>PaulR</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2195,16 +2308,23 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N38" t="n">
-        <v>2.5</v>
+        <v>17.31</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2225,12 +2345,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Harvey</t>
+          <t>Gerhart</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>PaytonL</t>
+          <t>PaulR</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -2239,16 +2359,23 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
       <c r="N39" t="n">
-        <v>2.5</v>
+        <v>15.88</v>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2269,12 +2396,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Harvey</t>
+          <t>Graves</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>PaytonL</t>
+          <t>CarsonJ</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -2283,20 +2410,19 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="n">
-        <v>17.31</v>
+        <v>2.5</v>
       </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2331,20 +2457,19 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>VISION</t>
-        </is>
-      </c>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="n">
-        <v>23</v>
+        <v>2.5</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2365,12 +2490,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>JeanLouis</t>
+          <t>Harvey</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Roody</t>
+          <t>PaytonL</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
@@ -2379,16 +2504,23 @@
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N42" t="n">
-        <v>2.5</v>
+        <v>17.31</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2409,12 +2541,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>LegaspiCisnero</t>
+          <t>Harvey</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>PaytonL</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2423,16 +2555,23 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
       <c r="N43" t="n">
-        <v>2.5</v>
+        <v>7.42</v>
       </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2453,12 +2592,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>LegaspiCisnero</t>
+          <t>Harvey</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>PaytonL</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2467,20 +2606,23 @@
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
-          <t>DENTAL</t>
+          <t>VISION</t>
         </is>
       </c>
       <c r="N44" t="n">
-        <v>17.31</v>
+        <v>23</v>
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2501,12 +2643,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>LegaspiCisnero</t>
+          <t>JeanLouis</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Roody</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2515,20 +2657,19 @@
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>VISION</t>
-        </is>
-      </c>
+      <c r="M45" t="inlineStr"/>
       <c r="N45" t="n">
-        <v>7.42</v>
+        <v>2.5</v>
       </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2549,12 +2690,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Malavet</t>
+          <t>LegaspiCisnero</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -2573,6 +2714,9 @@
       </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2593,12 +2737,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Massaad</t>
+          <t>LegaspiCisnero</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2607,16 +2751,23 @@
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N47" t="n">
-        <v>2.75</v>
+        <v>17.31</v>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2637,12 +2788,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mckee</t>
+          <t>LegaspiCisnero</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Maxwell</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
@@ -2651,16 +2802,23 @@
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
       <c r="N48" t="n">
-        <v>2.5</v>
+        <v>7.42</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2681,12 +2839,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mckee</t>
+          <t>Malavet</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Maxwell</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -2695,20 +2853,19 @@
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" t="n">
-        <v>17.31</v>
+        <v>2.5</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2729,12 +2886,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Mckee</t>
+          <t>Massaad</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Maxwell</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -2743,20 +2900,19 @@
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>VISION</t>
-        </is>
-      </c>
+      <c r="M50" t="inlineStr"/>
       <c r="N50" t="n">
-        <v>19.9</v>
+        <v>2.75</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2777,12 +2933,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Micenec</t>
+          <t>Mckee</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>MatthewR</t>
+          <t>Maxwell</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
@@ -2797,10 +2953,13 @@
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2821,12 +2980,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Noskey</t>
+          <t>Mckee</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Maxwell</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -2835,16 +2994,23 @@
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N52" t="n">
-        <v>2.5</v>
+        <v>17.31</v>
       </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2865,12 +3031,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Orr</t>
+          <t>Mckee</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Maxwell</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -2879,16 +3045,23 @@
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
       <c r="N53" t="n">
-        <v>2.75</v>
+        <v>19.9</v>
       </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2909,12 +3082,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Orr</t>
+          <t>Micenec</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>MatthewR</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -2923,20 +3096,19 @@
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M54" t="inlineStr"/>
       <c r="N54" t="n">
-        <v>17.31</v>
+        <v>4</v>
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2957,12 +3129,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Orr</t>
+          <t>Noskey</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Nicholas</t>
+          <t>Christian</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -2971,20 +3143,19 @@
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>VISION</t>
-        </is>
-      </c>
+      <c r="M55" t="inlineStr"/>
       <c r="N55" t="n">
-        <v>14.43</v>
+        <v>2.5</v>
       </c>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3005,12 +3176,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Ortiz-Hernandez</t>
+          <t>Orr</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Alfredo</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -3025,10 +3196,13 @@
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="n">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3049,12 +3223,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Ortiz-Hernandez</t>
+          <t>Orr</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Alfredo</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
@@ -3077,6 +3251,9 @@
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3097,12 +3274,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Ortiz-Hernandez</t>
+          <t>Orr</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Alfredo</t>
+          <t>Nicholas</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
@@ -3121,10 +3298,13 @@
         </is>
       </c>
       <c r="N58" t="n">
-        <v>12.74</v>
+        <v>14.43</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3145,12 +3325,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>PachecoMorillo</t>
+          <t>Ortiz-Hernandez</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Oscar</t>
+          <t>Alfredo</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -3159,20 +3339,19 @@
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M59" t="inlineStr"/>
       <c r="N59" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3193,12 +3372,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Proechel</t>
+          <t>Ortiz-Hernandez</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Greg</t>
+          <t>Alfredo</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
@@ -3207,16 +3386,23 @@
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N60" t="n">
-        <v>5.25</v>
+        <v>17.31</v>
       </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3237,12 +3423,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Proechel</t>
+          <t>Ortiz-Hernandez</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Greg</t>
+          <t>Alfredo</t>
         </is>
       </c>
       <c r="G61" t="inlineStr"/>
@@ -3251,20 +3437,23 @@
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
-          <t>DENTAL</t>
+          <t>VISION</t>
         </is>
       </c>
       <c r="N61" t="n">
-        <v>17.31</v>
+        <v>12.74</v>
       </c>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3285,12 +3474,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Proechel</t>
+          <t>PachecoMorillo</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Greg</t>
+          <t>Oscar</t>
         </is>
       </c>
       <c r="G62" t="inlineStr"/>
@@ -3299,20 +3488,23 @@
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr">
         <is>
-          <t>VISION</t>
+          <t>DENTAL</t>
         </is>
       </c>
       <c r="N62" t="n">
-        <v>7.42</v>
+        <v>4</v>
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3333,12 +3525,12 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Rodriguez</t>
+          <t>Proechel</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>KristianL</t>
+          <t>Greg</t>
         </is>
       </c>
       <c r="G63" t="inlineStr"/>
@@ -3347,20 +3539,19 @@
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M63" t="inlineStr"/>
       <c r="N63" t="n">
-        <v>2.5</v>
+        <v>5.25</v>
       </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3381,12 +3572,12 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Sarmiento</t>
+          <t>Proechel</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>DanielA</t>
+          <t>Greg</t>
         </is>
       </c>
       <c r="G64" t="inlineStr"/>
@@ -3395,16 +3586,23 @@
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N64" t="n">
-        <v>2.5</v>
+        <v>17.31</v>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3425,12 +3623,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Sarmiento</t>
+          <t>Proechel</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>DanielA</t>
+          <t>Greg</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
@@ -3439,20 +3637,23 @@
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
-          <t>DENTAL</t>
+          <t>VISION</t>
         </is>
       </c>
       <c r="N65" t="n">
-        <v>17.31</v>
+        <v>7.42</v>
       </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3473,12 +3674,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Sarmiento</t>
+          <t>Proechel</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>DanielA</t>
+          <t>Greg</t>
         </is>
       </c>
       <c r="G66" t="inlineStr"/>
@@ -3487,20 +3688,19 @@
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>TotalPremium</t>
         </is>
       </c>
       <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>VISION</t>
-        </is>
-      </c>
+      <c r="M66" t="inlineStr"/>
       <c r="N66" t="n">
-        <v>7.42</v>
+        <v>55.07</v>
       </c>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3521,12 +3721,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Stealey</t>
+          <t>Rodriguez</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Eric</t>
+          <t>KristianL</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
@@ -3535,16 +3735,23 @@
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N67" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3565,12 +3772,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Stealey</t>
+          <t>Sarmiento</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Eric</t>
+          <t>DanielA</t>
         </is>
       </c>
       <c r="G68" t="inlineStr"/>
@@ -3579,20 +3786,19 @@
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M68" t="inlineStr"/>
       <c r="N68" t="n">
-        <v>17.31</v>
+        <v>2.5</v>
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3613,12 +3819,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Tovar</t>
+          <t>Sarmiento</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Frank</t>
+          <t>DanielA</t>
         </is>
       </c>
       <c r="G69" t="inlineStr"/>
@@ -3627,16 +3833,23 @@
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
       <c r="N69" t="n">
-        <v>44</v>
+        <v>17.31</v>
       </c>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3657,12 +3870,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Tovar</t>
+          <t>Sarmiento</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Frank</t>
+          <t>DanielA</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
@@ -3671,20 +3884,23 @@
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>Vision</t>
         </is>
       </c>
       <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
-          <t>DENTAL</t>
+          <t>VISION</t>
         </is>
       </c>
       <c r="N70" t="n">
-        <v>17.31</v>
+        <v>7.42</v>
       </c>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3705,12 +3921,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Winters</t>
+          <t>Sarmiento</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Mitchell</t>
+          <t>DanielA</t>
         </is>
       </c>
       <c r="G71" t="inlineStr"/>
@@ -3719,16 +3935,19 @@
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
-          <t>BasicTermLife</t>
+          <t>TotalPremium</t>
         </is>
       </c>
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="n">
-        <v>2.5</v>
+        <v>39.93</v>
       </c>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3749,12 +3968,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Winters</t>
+          <t>Stealey</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Mitchell</t>
+          <t>Eric</t>
         </is>
       </c>
       <c r="G72" t="inlineStr"/>
@@ -3763,20 +3982,19 @@
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M72" t="inlineStr"/>
       <c r="N72" t="n">
-        <v>17.31</v>
+        <v>2.75</v>
       </c>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3797,12 +4015,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Winters</t>
+          <t>Stealey</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Mitchell</t>
+          <t>Eric</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
@@ -3811,20 +4029,23 @@
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Vision</t>
+          <t>Dental</t>
         </is>
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
-          <t>VISION</t>
+          <t>DENTAL</t>
         </is>
       </c>
       <c r="N73" t="n">
-        <v>7.42</v>
+        <v>17.31</v>
       </c>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3845,12 +4066,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Yoder</t>
+          <t>Stealey</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>GaryM</t>
+          <t>Eric</t>
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
@@ -3859,20 +4080,19 @@
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>TotalPremium</t>
         </is>
       </c>
       <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M74" t="inlineStr"/>
       <c r="N74" t="n">
-        <v>2.5</v>
+        <v>35.94</v>
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="n">
+        <v>709.78</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3893,12 +4113,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Zwetsch</t>
+          <t>Tovar</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Ryan</t>
+          <t>Frank</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
@@ -3907,20 +4127,415 @@
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Dental</t>
+          <t>BasicTermLife</t>
         </is>
       </c>
       <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>DENTAL</t>
-        </is>
-      </c>
+      <c r="M75" t="inlineStr"/>
       <c r="N75" t="n">
-        <v>2.5</v>
+        <v>44</v>
       </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Tovar</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Frank</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>17.31</v>
+      </c>
+      <c r="O76" t="inlineStr"/>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Tovar</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Frank</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>TotalPremium</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="O77" t="inlineStr"/>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Winters</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Mitchell</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>BasicTermLife</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O78" t="inlineStr"/>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Winters</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Mitchell</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
+        <v>17.31</v>
+      </c>
+      <c r="O79" t="inlineStr"/>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Winters</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Mitchell</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Vision</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>VISION</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="O80" t="inlineStr"/>
+      <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Winters</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Mitchell</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>TotalPremium</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
+      <c r="N81" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr"/>
+      <c r="Q81" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Yoder</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>GaryM</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="n">
+        <v>709.78</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Guardian Rocca Feb-25 Inv 2.pdf</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>01/17/25</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>02/01/25 to 02/28/25</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Zwetsch</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Dental</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>DENTAL</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O83" t="inlineStr"/>
+      <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="n">
+        <v>709.78</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>